<commit_message>
update monthly visits output
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/Output_monthly_visits_Raw.xlsx
+++ b/CPRD Raw Analysis/Results/Output_monthly_visits_Raw.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -368,25 +368,35 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>sd_visits</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>q1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>median</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>q3</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>n_pts</t>
         </is>
@@ -397,22 +407,28 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>3.09</v>
+        <v>3.08</v>
       </c>
       <c r="C2">
-        <v>2.41</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
         <v>4</v>
       </c>
-      <c r="G2">
-        <v>19299</v>
+      <c r="I2">
+        <v>19034</v>
       </c>
     </row>
     <row r="3">
@@ -423,19 +439,25 @@
         <v>2.68</v>
       </c>
       <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>25</v>
+      </c>
+      <c r="E3">
         <v>2.22</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>15876</v>
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>15872</v>
       </c>
     </row>
     <row r="4">
@@ -446,18 +468,24 @@
         <v>2.64</v>
       </c>
       <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>36</v>
+      </c>
+      <c r="E4">
         <v>2.2</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
       <c r="F4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4">
         <v>14615</v>
       </c>
     </row>
@@ -469,18 +497,24 @@
         <v>2.54</v>
       </c>
       <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>32</v>
+      </c>
+      <c r="E5">
         <v>2.08</v>
       </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
       <c r="F5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="I5">
         <v>13625</v>
       </c>
     </row>
@@ -492,18 +526,24 @@
         <v>2.53</v>
       </c>
       <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>34</v>
+      </c>
+      <c r="E6">
         <v>2.12</v>
       </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
       <c r="F6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
         <v>12723</v>
       </c>
     </row>
@@ -515,18 +555,24 @@
         <v>2.49</v>
       </c>
       <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>24</v>
+      </c>
+      <c r="E7">
         <v>2.05</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>2</v>
-      </c>
       <c r="F7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7">
         <v>12233</v>
       </c>
     </row>
@@ -538,18 +584,24 @@
         <v>2.48</v>
       </c>
       <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="E8">
         <v>2.03</v>
       </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
       <c r="F8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8">
+        <v>3</v>
+      </c>
+      <c r="I8">
         <v>11695</v>
       </c>
     </row>
@@ -561,18 +613,24 @@
         <v>2.42</v>
       </c>
       <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9">
         <v>1.98</v>
       </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>2</v>
-      </c>
       <c r="F9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+      <c r="I9">
         <v>11347</v>
       </c>
     </row>
@@ -584,18 +642,24 @@
         <v>2.48</v>
       </c>
       <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>32</v>
+      </c>
+      <c r="E10">
         <v>2.03</v>
       </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>2</v>
-      </c>
       <c r="F10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G10">
+        <v>2</v>
+      </c>
+      <c r="H10">
+        <v>3</v>
+      </c>
+      <c r="I10">
         <v>11155</v>
       </c>
     </row>
@@ -607,18 +671,24 @@
         <v>2.42</v>
       </c>
       <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>34</v>
+      </c>
+      <c r="E11">
         <v>1.96</v>
       </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>2</v>
-      </c>
       <c r="F11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11">
+        <v>2</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
+      </c>
+      <c r="I11">
         <v>10900</v>
       </c>
     </row>
@@ -630,18 +700,24 @@
         <v>2.42</v>
       </c>
       <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>42</v>
+      </c>
+      <c r="E12">
         <v>1.97</v>
       </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12">
-        <v>2</v>
-      </c>
       <c r="F12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G12">
+        <v>2</v>
+      </c>
+      <c r="H12">
+        <v>3</v>
+      </c>
+      <c r="I12">
         <v>10696</v>
       </c>
     </row>
@@ -653,18 +729,24 @@
         <v>2.45</v>
       </c>
       <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>32</v>
+      </c>
+      <c r="E13">
         <v>2.01</v>
       </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13">
-        <v>2</v>
-      </c>
       <c r="F13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>3</v>
+      </c>
+      <c r="I13">
         <v>10585</v>
       </c>
     </row>
@@ -676,18 +758,24 @@
         <v>2.44</v>
       </c>
       <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>30</v>
+      </c>
+      <c r="E14">
         <v>1.96</v>
       </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14">
-        <v>2</v>
-      </c>
       <c r="F14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G14">
+        <v>2</v>
+      </c>
+      <c r="H14">
+        <v>3</v>
+      </c>
+      <c r="I14">
         <v>10438</v>
       </c>
     </row>
@@ -699,18 +787,24 @@
         <v>2.44</v>
       </c>
       <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>21</v>
+      </c>
+      <c r="E15">
         <v>1.97</v>
       </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-      <c r="E15">
-        <v>2</v>
-      </c>
       <c r="F15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
         <v>10096</v>
       </c>
     </row>
@@ -722,18 +816,24 @@
         <v>2.48</v>
       </c>
       <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>23</v>
+      </c>
+      <c r="E16">
         <v>2.04</v>
       </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16">
-        <v>2</v>
-      </c>
       <c r="F16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G16">
+        <v>2</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
         <v>9940</v>
       </c>
     </row>
@@ -745,18 +845,24 @@
         <v>2.42</v>
       </c>
       <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>28</v>
+      </c>
+      <c r="E17">
         <v>1.98</v>
       </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17">
-        <v>2</v>
-      </c>
       <c r="F17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G17">
+        <v>2</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
         <v>9820</v>
       </c>
     </row>
@@ -768,18 +874,24 @@
         <v>2.43</v>
       </c>
       <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>28</v>
+      </c>
+      <c r="E18">
         <v>1.95</v>
       </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
-      <c r="E18">
-        <v>2</v>
-      </c>
       <c r="F18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G18">
+        <v>2</v>
+      </c>
+      <c r="H18">
+        <v>3</v>
+      </c>
+      <c r="I18">
         <v>9735</v>
       </c>
     </row>
@@ -791,18 +903,24 @@
         <v>2.44</v>
       </c>
       <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>23</v>
+      </c>
+      <c r="E19">
         <v>2.02</v>
       </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
-      <c r="E19">
-        <v>2</v>
-      </c>
       <c r="F19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19">
+        <v>3</v>
+      </c>
+      <c r="I19">
         <v>9606</v>
       </c>
     </row>
@@ -814,18 +932,24 @@
         <v>2.41</v>
       </c>
       <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>25</v>
+      </c>
+      <c r="E20">
         <v>1.96</v>
       </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20">
-        <v>2</v>
-      </c>
       <c r="F20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20">
+        <v>3</v>
+      </c>
+      <c r="I20">
         <v>9591</v>
       </c>
     </row>
@@ -837,18 +961,24 @@
         <v>2.43</v>
       </c>
       <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>26</v>
+      </c>
+      <c r="E21">
         <v>1.99</v>
       </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21">
-        <v>2</v>
-      </c>
       <c r="F21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21">
+        <v>3</v>
+      </c>
+      <c r="I21">
         <v>9411</v>
       </c>
     </row>
@@ -860,18 +990,24 @@
         <v>2.43</v>
       </c>
       <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>21</v>
+      </c>
+      <c r="E22">
         <v>1.98</v>
       </c>
-      <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22">
-        <v>2</v>
-      </c>
       <c r="F22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="H22">
+        <v>3</v>
+      </c>
+      <c r="I22">
         <v>9332</v>
       </c>
     </row>
@@ -883,18 +1019,24 @@
         <v>2.41</v>
       </c>
       <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>22</v>
+      </c>
+      <c r="E23">
         <v>1.93</v>
       </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23">
-        <v>2</v>
-      </c>
       <c r="F23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="H23">
+        <v>3</v>
+      </c>
+      <c r="I23">
         <v>9113</v>
       </c>
     </row>
@@ -906,18 +1048,24 @@
         <v>2.41</v>
       </c>
       <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>20</v>
+      </c>
+      <c r="E24">
         <v>1.93</v>
       </c>
-      <c r="D24">
-        <v>1</v>
-      </c>
-      <c r="E24">
-        <v>2</v>
-      </c>
       <c r="F24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G24">
+        <v>2</v>
+      </c>
+      <c r="H24">
+        <v>3</v>
+      </c>
+      <c r="I24">
         <v>9107</v>
       </c>
     </row>
@@ -929,18 +1077,24 @@
         <v>2.41</v>
       </c>
       <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>19</v>
+      </c>
+      <c r="E25">
         <v>1.96</v>
       </c>
-      <c r="D25">
-        <v>1</v>
-      </c>
-      <c r="E25">
-        <v>2</v>
-      </c>
       <c r="F25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G25">
+        <v>2</v>
+      </c>
+      <c r="H25">
+        <v>3</v>
+      </c>
+      <c r="I25">
         <v>8906</v>
       </c>
     </row>
@@ -952,18 +1106,24 @@
         <v>1.07</v>
       </c>
       <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>3</v>
+      </c>
+      <c r="E26">
         <v>0.27</v>
       </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="E26">
-        <v>1</v>
-      </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
         <v>405</v>
       </c>
     </row>
@@ -974,7 +1134,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -990,25 +1150,35 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>sd_visits</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>q1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>median</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>q3</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>n_pts</t>
         </is>
@@ -1019,22 +1189,28 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>3.09</v>
+        <v>3.08</v>
       </c>
       <c r="C2">
-        <v>2.41</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
         <v>4</v>
       </c>
-      <c r="G2">
-        <v>19193</v>
+      <c r="I2">
+        <v>19034</v>
       </c>
     </row>
     <row r="3">
@@ -1045,18 +1221,24 @@
         <v>2.68</v>
       </c>
       <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>25</v>
+      </c>
+      <c r="E3">
         <v>2.23</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3">
         <v>15793</v>
       </c>
     </row>
@@ -1068,18 +1250,24 @@
         <v>2.64</v>
       </c>
       <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>36</v>
+      </c>
+      <c r="E4">
         <v>2.2</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
       <c r="F4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4">
         <v>14544</v>
       </c>
     </row>
@@ -1091,18 +1279,24 @@
         <v>2.55</v>
       </c>
       <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>32</v>
+      </c>
+      <c r="E5">
         <v>2.08</v>
       </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
       <c r="F5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="I5">
         <v>13433</v>
       </c>
     </row>
@@ -1114,18 +1308,24 @@
         <v>2.54</v>
       </c>
       <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>34</v>
+      </c>
+      <c r="E6">
         <v>2.12</v>
       </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
       <c r="F6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
         <v>12599</v>
       </c>
     </row>
@@ -1137,18 +1337,24 @@
         <v>2.49</v>
       </c>
       <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>24</v>
+      </c>
+      <c r="E7">
         <v>2.06</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>2</v>
-      </c>
       <c r="F7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7">
         <v>12120</v>
       </c>
     </row>
@@ -1160,18 +1366,24 @@
         <v>2.48</v>
       </c>
       <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="E8">
         <v>2.03</v>
       </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
       <c r="F8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8">
+        <v>3</v>
+      </c>
+      <c r="I8">
         <v>11620</v>
       </c>
     </row>
@@ -1183,18 +1395,24 @@
         <v>2.43</v>
       </c>
       <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9">
         <v>1.99</v>
       </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>2</v>
-      </c>
       <c r="F9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+      <c r="I9">
         <v>11261</v>
       </c>
     </row>
@@ -1206,18 +1424,24 @@
         <v>2.48</v>
       </c>
       <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>32</v>
+      </c>
+      <c r="E10">
         <v>2.03</v>
       </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>2</v>
-      </c>
       <c r="F10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G10">
+        <v>2</v>
+      </c>
+      <c r="H10">
+        <v>3</v>
+      </c>
+      <c r="I10">
         <v>11084</v>
       </c>
     </row>
@@ -1229,18 +1453,24 @@
         <v>2.43</v>
       </c>
       <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>34</v>
+      </c>
+      <c r="E11">
         <v>1.96</v>
       </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>2</v>
-      </c>
       <c r="F11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11">
+        <v>2</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
+      </c>
+      <c r="I11">
         <v>10842</v>
       </c>
     </row>
@@ -1252,18 +1482,24 @@
         <v>2.43</v>
       </c>
       <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>42</v>
+      </c>
+      <c r="E12">
         <v>1.97</v>
       </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12">
-        <v>2</v>
-      </c>
       <c r="F12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G12">
+        <v>2</v>
+      </c>
+      <c r="H12">
+        <v>3</v>
+      </c>
+      <c r="I12">
         <v>10638</v>
       </c>
     </row>
@@ -1275,18 +1511,24 @@
         <v>2.45</v>
       </c>
       <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>32</v>
+      </c>
+      <c r="E13">
         <v>2.01</v>
       </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13">
-        <v>2</v>
-      </c>
       <c r="F13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>3</v>
+      </c>
+      <c r="I13">
         <v>10523</v>
       </c>
     </row>
@@ -1298,18 +1540,24 @@
         <v>2.44</v>
       </c>
       <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>30</v>
+      </c>
+      <c r="E14">
         <v>1.97</v>
       </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14">
-        <v>2</v>
-      </c>
       <c r="F14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G14">
+        <v>2</v>
+      </c>
+      <c r="H14">
+        <v>3</v>
+      </c>
+      <c r="I14">
         <v>10386</v>
       </c>
     </row>
@@ -1321,18 +1569,24 @@
         <v>2.44</v>
       </c>
       <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>21</v>
+      </c>
+      <c r="E15">
         <v>1.97</v>
       </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-      <c r="E15">
-        <v>2</v>
-      </c>
       <c r="F15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
         <v>10054</v>
       </c>
     </row>
@@ -1344,18 +1598,24 @@
         <v>2.48</v>
       </c>
       <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>23</v>
+      </c>
+      <c r="E16">
         <v>2.04</v>
       </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16">
-        <v>2</v>
-      </c>
       <c r="F16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G16">
+        <v>2</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
         <v>9895</v>
       </c>
     </row>
@@ -1367,18 +1627,24 @@
         <v>2.42</v>
       </c>
       <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>28</v>
+      </c>
+      <c r="E17">
         <v>1.97</v>
       </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17">
-        <v>2</v>
-      </c>
       <c r="F17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G17">
+        <v>2</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
         <v>9771</v>
       </c>
     </row>
@@ -1390,18 +1656,24 @@
         <v>2.43</v>
       </c>
       <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>28</v>
+      </c>
+      <c r="E18">
         <v>1.95</v>
       </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
-      <c r="E18">
-        <v>2</v>
-      </c>
       <c r="F18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G18">
+        <v>2</v>
+      </c>
+      <c r="H18">
+        <v>3</v>
+      </c>
+      <c r="I18">
         <v>9692</v>
       </c>
     </row>
@@ -1413,18 +1685,24 @@
         <v>2.44</v>
       </c>
       <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>23</v>
+      </c>
+      <c r="E19">
         <v>2.03</v>
       </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
-      <c r="E19">
-        <v>2</v>
-      </c>
       <c r="F19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19">
+        <v>3</v>
+      </c>
+      <c r="I19">
         <v>9561</v>
       </c>
     </row>
@@ -1436,18 +1714,24 @@
         <v>2.41</v>
       </c>
       <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>25</v>
+      </c>
+      <c r="E20">
         <v>1.96</v>
       </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20">
-        <v>2</v>
-      </c>
       <c r="F20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20">
+        <v>3</v>
+      </c>
+      <c r="I20">
         <v>9552</v>
       </c>
     </row>
@@ -1459,18 +1743,24 @@
         <v>2.43</v>
       </c>
       <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>26</v>
+      </c>
+      <c r="E21">
         <v>1.99</v>
       </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21">
-        <v>2</v>
-      </c>
       <c r="F21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21">
+        <v>3</v>
+      </c>
+      <c r="I21">
         <v>9369</v>
       </c>
     </row>
@@ -1482,18 +1772,24 @@
         <v>2.43</v>
       </c>
       <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>21</v>
+      </c>
+      <c r="E22">
         <v>1.98</v>
       </c>
-      <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22">
-        <v>2</v>
-      </c>
       <c r="F22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="H22">
+        <v>3</v>
+      </c>
+      <c r="I22">
         <v>9293</v>
       </c>
     </row>
@@ -1505,18 +1801,24 @@
         <v>2.41</v>
       </c>
       <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>22</v>
+      </c>
+      <c r="E23">
         <v>1.94</v>
       </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23">
-        <v>2</v>
-      </c>
       <c r="F23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="H23">
+        <v>3</v>
+      </c>
+      <c r="I23">
         <v>9066</v>
       </c>
     </row>
@@ -1528,18 +1830,24 @@
         <v>2.42</v>
       </c>
       <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>20</v>
+      </c>
+      <c r="E24">
         <v>1.93</v>
       </c>
-      <c r="D24">
-        <v>1</v>
-      </c>
-      <c r="E24">
-        <v>2</v>
-      </c>
       <c r="F24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G24">
+        <v>2</v>
+      </c>
+      <c r="H24">
+        <v>3</v>
+      </c>
+      <c r="I24">
         <v>9079</v>
       </c>
     </row>
@@ -1551,18 +1859,24 @@
         <v>2.42</v>
       </c>
       <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>19</v>
+      </c>
+      <c r="E25">
         <v>1.96</v>
       </c>
-      <c r="D25">
-        <v>1</v>
-      </c>
-      <c r="E25">
-        <v>2</v>
-      </c>
       <c r="F25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G25">
+        <v>2</v>
+      </c>
+      <c r="H25">
+        <v>3</v>
+      </c>
+      <c r="I25">
         <v>8866</v>
       </c>
     </row>
@@ -1574,18 +1888,24 @@
         <v>1</v>
       </c>
       <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
         <v>0</v>
       </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="E26">
-        <v>1</v>
-      </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
         <v>9</v>
       </c>
     </row>

</xml_diff>